<commit_message>
Update protocol: restructured introduction, Table 12 summary comparison, rho variance-components figure, small-study-effect caveats, and various citation/wording fixes
</commit_message>
<xml_diff>
--- a/Table5S_Protocol.xlsx
+++ b/Table5S_Protocol.xlsx
@@ -1,41 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Panel A - No controls" sheetId="1" r:id="rId1"/>
-    <sheet name="Panel B - Full controls" sheetId="2" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel A - No controls" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel B - Full controls" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -54,16 +55,83 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -351,11 +419,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
+    <row r="1" customFormat="1" s="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Variable</t>
@@ -582,7 +654,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tau</t>
+          <t>rho (assumed)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -592,29 +664,29 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.171</t>
+          <t>--</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.130</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.118</t>
+          <t>--</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.077</t>
+          <t>0.500</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>omega</t>
+          <t>tau</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -624,52 +696,84 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>0.171</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>0.130</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.147</t>
+          <t>0.118</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.157</t>
+          <t>0.077</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>omega</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0.147</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.157</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>LR test</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>p &lt; .0001</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>p &lt; .0001</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>p &lt; .0001</t>
         </is>
@@ -681,11 +785,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
+    <row r="1" customFormat="1" s="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Variable</t>
@@ -912,7 +1020,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tau</t>
+          <t>rho (assumed)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -922,29 +1030,29 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.160</t>
+          <t>--</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.138</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.130</t>
+          <t>--</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.091</t>
+          <t>0.500</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>omega</t>
+          <t>tau</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -954,52 +1062,84 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>0.160</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>--</t>
+          <t>0.138</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.142</t>
+          <t>0.130</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.153</t>
+          <t>0.091</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>omega</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>0.142</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.153</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>LR test</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>p &lt; .0001</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>--</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>p &lt; .0001</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>p &lt; .0001</t>
         </is>

</xml_diff>